<commit_message>
Motherson PKC Update: 📦 Warehouse
</commit_message>
<xml_diff>
--- a/02_Warehouse_Stock_Alert.xlsx
+++ b/02_Warehouse_Stock_Alert.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,15 +454,45 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>Stock Status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Reorder Point</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Daily Consumption</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Estimated Stock-Out Date</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Lifecycle Stage</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Warehouse Location</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
@@ -496,11 +526,37 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-21 17:05</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+          <t>🟢 Normal Stock</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>🟢 Normal</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Alert Created</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:16</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -530,11 +586,37 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-21 17:05</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+          <t>🔴 Shortage</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>🚨 Critical</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>20</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-12-12</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Alert Created</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:16</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Motherson PKC Add row in 📦 Warehouse
</commit_message>
<xml_diff>
--- a/02_Warehouse_Stock_Alert.xlsx
+++ b/02_Warehouse_Stock_Alert.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,7 +552,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-23 10:16</t>
+          <t>2026-09-21 17:20</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -612,11 +612,71 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-23 10:16</t>
+          <t>2026-09-21 17:20</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ALT-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TEST-003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" t="n">
+        <v>90</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>🔴 Shortage</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>🚨 Critical</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>25</v>
+      </c>
+      <c r="K4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Alert Created</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-09-23 10:17</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add product ALT-005 in 📦 Warehouse
</commit_message>
<xml_diff>
--- a/02_Warehouse_Stock_Alert.xlsx
+++ b/02_Warehouse_Stock_Alert.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,7 +591,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>🚨 ALERT: 🔴 Shortage (Shortage/Diff: 100.0 units)</t>
+          <t>🚨 ALERT: 🔴 Shortage (Shortage: 100.0 units)</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -783,7 +783,7 @@
         <v>230</v>
       </c>
       <c r="G4" t="n">
-        <v>-180</v>
+        <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
         <v>11</v>
       </c>
       <c r="G5" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -941,6 +941,65 @@
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ALT-ALT-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ALT-005</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-09-23 15:25</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Full system sync from 🏭 Production Department
</commit_message>
<xml_diff>
--- a/02_Warehouse_Stock_Alert.xlsx
+++ b/02_Warehouse_Stock_Alert.xlsx
@@ -556,42 +556,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ALT-003</t>
+          <t>ALT-002</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TEST-003</t>
+          <t>TEST-002</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="F2" t="n">
-        <v>230</v>
+        <v>400</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>🟢 Normal Stock</t>
+          <t>🔴 Shortage</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>🟢 Normal</t>
+          <t>🚨 Critical</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>✅ Normal (Stock OK)</t>
+          <t>🚨 ALERT: 🔴 Shortage (Shortage: 100 units)</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -601,24 +601,24 @@
         <v>5</v>
       </c>
       <c r="M2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N2" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>No Reorder</t>
+          <t>No Reorder Required</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-23 15:25</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -641,7 +641,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>PO-TEST-003</t>
+          <t>PO-TEST-002</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -659,28 +659,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ALT-002</t>
+          <t>ALT-ALT-005</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TEST-002</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>ALT-005</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
       <c r="E3" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -694,11 +696,11 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>🚨 ALERT: 🔴 Shortage (Shortage: 100.0 units)</t>
+          <t>🚨 ALERT: 🔴 Shortage (Shortage: 99 units)</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
         <v>5</v>
@@ -707,57 +709,33 @@
         <v>10</v>
       </c>
       <c r="N3" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>No Reorder</t>
+          <t>Reorder Triggered</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-23 15:25</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Default Supplier</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>PO-TEST-002</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Road</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>In Transit</t>
-        </is>
-      </c>
+      <c r="AA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -814,7 +792,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Reorder Required</t>
+          <t>Reorder Triggered</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -824,7 +802,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-23 15:25</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -841,7 +819,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ALT-ALT-005</t>
+          <t>ALT-003</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -851,73 +829,95 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ALT-005</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
+          <t>TEST-003</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>230</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>🔴 Last Box</t>
+          <t>🟢 Normal Stock</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>🔴 High</t>
+          <t>🟢 Normal</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>🚨 ALERT: 🔴 Last Box (Shortage: 0.0 units)</t>
+          <t>✅ Normal (Stock Optimal)</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
         <v>5</v>
       </c>
       <c r="M5" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N5" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Reorder Required</t>
+          <t>No Reorder Required</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-09-23 15:25</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Default Supplier</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>PO-TEST-003</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Road</t>
+        </is>
+      </c>
       <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>✅ Normal (Stock OK)</t>
+          <t>✅ Normal (Stock Optimal)</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -974,7 +974,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>No Reorder</t>
+          <t>No Reorder Required</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-09-23 15:25</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R6" t="inlineStr"/>

</xml_diff>